<commit_message>
docs: expand My Orders test cases to 25 scenarios
</commit_message>
<xml_diff>
--- a/Test cases of Globewest/Sprint 3 - My Order Page Test Cases.xlsx
+++ b/Test cases of Globewest/Sprint 3 - My Order Page Test Cases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
+    <sheet name="My Orders Test Cases" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,18 +397,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J26"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="42.83203125" customWidth="1"/>
     <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="64.83203125" customWidth="1"/>
-    <col min="5" max="5" width="64.83203125" customWidth="1"/>
-    <col min="6" max="6" width="64.83203125" customWidth="1"/>
-    <col min="7" max="7" width="64.83203125" customWidth="1"/>
-    <col min="8" max="8" width="64.83203125" customWidth="1"/>
-    <col min="9" max="9" width="34.83203125" customWidth="1"/>
-    <col min="10" max="10" width="29.83203125" customWidth="1"/>
+    <col min="4" max="4" width="54.83203125" customWidth="1"/>
+    <col min="5" max="5" width="54.83203125" customWidth="1"/>
+    <col min="6" max="6" width="54.83203125" customWidth="1"/>
+    <col min="7" max="7" width="54.83203125" customWidth="1"/>
+    <col min="8" max="8" width="54.83203125" customWidth="1"/>
+    <col min="9" max="9" width="12.83203125" customWidth="1"/>
+    <col min="10" max="10" width="12.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -462,7 +462,7 @@
       <c r="F2" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Navigate to customer login page (/customer/account/login/)
 2. Enter valid Trade Customer credentials
-3. Click 'Sign In'
+3. Click "Sign In"
 4. Navigate to My Orders URL (/gw_orders/order/index/)</v>
       </c>
       <c r="G2" t="str">
@@ -475,7 +475,7 @@
         <v>PASS</v>
       </c>
       <c r="J2" t="str">
-        <v>LOW (Core Route Verified)</v>
+        <v>LOW</v>
       </c>
     </row>
     <row r="3" xml:space="preserve">
@@ -489,7 +489,7 @@
         <v>Trade Customer (Logged In)</v>
       </c>
       <c r="D3" t="str">
-        <v>Verify Default Active Status Filter Tab is 'AWAITING PAYMENT' (Frame 624 Rule 1)</v>
+        <v>Verify Default Active Status Filter Tab is "AWAITING PAYMENT" (Frame 624 Rule 1)</v>
       </c>
       <c r="E3" t="str">
         <v>Logged-in Trade Customer accessing clean session on /gw_orders/order/index/</v>
@@ -500,10 +500,10 @@
 3. Inspect which tab is highlighted and active by default</v>
       </c>
       <c r="G3" t="str">
-        <v>Per Frame 624: 'Tabs that filter table view of orders shown based on status. Default to awaiting payment'. Active tab must default to 'AWAITING PAYMENT' with solid dark pill styling (#2B1D16).</v>
+        <v>Per Frame 624: "Tabs that filter table view of orders shown based on status. Default to awaiting payment". Active tab must default to "AWAITING PAYMENT" with solid dark pill styling (#2B1D16).</v>
       </c>
       <c r="H3" t="str">
-        <v>Page erroneously defaults to the 'OPEN' tab with a plain text underline. 'AWAITING PAYMENT' tab is missing.</v>
+        <v>Page erroneously defaults to the "OPEN" tab with a plain text underline. "AWAITING PAYMENT" tab is missing.</v>
       </c>
       <c r="I3" t="str">
         <v>FAIL</v>
@@ -537,7 +537,7 @@
         <v>Render 4 segmented tabs: [ AWAITING PAYMENT ] [ PENDING SHIPMENT ] [ DISPATCHED ] [ CLOSED ]. Pills have capsule shape and active dark fill.</v>
       </c>
       <c r="H4" t="str">
-        <v>Only renders 3 tabs: 'ALL', 'OPEN', 'CLOSED'. Tabs are unstyled plain text links. Missing 'PENDING SHIPMENT' and 'DISPATCHED'.</v>
+        <v>Only renders 3 tabs: "ALL", "OPEN", "CLOSED". Tabs are unstyled plain text links. Missing "PENDING SHIPMENT" and "DISPATCHED".</v>
       </c>
       <c r="I4" t="str">
         <v>FAIL</v>
@@ -568,7 +568,7 @@
 3. Verify column header labels.</v>
       </c>
       <c r="G5" t="str">
-        <v>Per Frame 624: 'Reduction of columns shown'. Exactly 6 columns: ORDER ⬍, DATE ⬍, STATUS ⬍, TOTAL ⬍, BALANCE ⬍, ACTIONS.</v>
+        <v>Per Frame 624: "Reduction of columns shown". Exactly 6 columns: ORDER ⬍, DATE ⬍, STATUS ⬍, TOTAL ⬍, BALANCE ⬍, ACTIONS.</v>
       </c>
       <c r="H5" t="str">
         <v>Live staging displays 10 columns: Order, Date, Cust po#, Order name, Client Name, Status, Total, Balance, Details, Actions.</v>
@@ -597,14 +597,14 @@
         <v>Logged-in Trade Customer on /gw_orders/order/index/</v>
       </c>
       <c r="F6" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Verify whether a separate 'DETAILS' header/column exists.
-2. Verify presence of 'Cust po#', 'Order name', 'Client Name'.</v>
+        <v xml:space="preserve">1. Verify whether a separate "DETAILS" header/column exists.
+2. Verify presence of "Cust po#", "Order name", "Client Name".</v>
       </c>
       <c r="G6" t="str">
-        <v>No standalone 'DETAILS' column. No 'Cust po#', 'Order name', or 'Client Name' columns in default grid.</v>
+        <v>No standalone "DETAILS" column. No "Cust po#", "Order name", or "Client Name" columns in default grid.</v>
       </c>
       <c r="H6" t="str">
-        <v>Redundant unstyled 'DETAILS' column is rendered alongside separate 'ACTIONS' column, plus 3 redundant metadata columns.</v>
+        <v>Redundant unstyled "DETAILS" column is rendered alongside separate "ACTIONS" column, plus 3 redundant metadata columns.</v>
       </c>
       <c r="I6" t="str">
         <v>FAIL</v>
@@ -635,13 +635,13 @@
 3. Observe destination URL and rendered view.</v>
       </c>
       <c r="G7" t="str">
-        <v>Per Frame 624: 'Order number to be linked + clickable to the order details page'. Clicking order # navigates to /gw_orders/order/view/order_id/X/.</v>
+        <v>Per Frame 624: "Order number to be linked + clickable to the order details page". Clicking order # navigates to /gw_orders/order/view/order_id/X/.</v>
       </c>
       <c r="H7" t="str">
-        <v>Must verify clickable hyperlink presence once test data / dev build is deployed.</v>
+        <v>Order number is rendered as a clickable link leading directly to the Order Details page.</v>
       </c>
       <c r="I7" t="str">
-        <v>TO VERIFY (Awaiting Data)</v>
+        <v>PASS</v>
       </c>
       <c r="J7" t="str">
         <v>HIGH</v>
@@ -658,18 +658,18 @@
         <v>Trade Customer (Logged In)</v>
       </c>
       <c r="D8" t="str">
-        <v>Verify Unified 'Actions ▾' Dropdown on Desktop &amp; Mobile (Frame 624 Rule 3)</v>
+        <v>Verify Unified "Actions ▾" Dropdown on Desktop &amp; Mobile (Frame 624 Rule 3)</v>
       </c>
       <c r="E8" t="str">
         <v>Orders grid populated with order records</v>
       </c>
       <c r="F8" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Locate 'ACTIONS' column on each row.
-2. Click 'Actions ▾' dropdown button.
+        <v xml:space="preserve">1. Locate "ACTIONS" column on each row.
+2. Click "Actions ▾" dropdown button.
 3. Verify menu options (View Order, Reorder, Print Invoice).</v>
       </c>
       <c r="G8" t="str">
-        <v>Per Frame 624: 'Actions housed under dropdown for both mobile + desktop as per other table functionality'. Clean consolidated dropdown on every row.</v>
+        <v>Per Frame 624: "Actions housed under dropdown for both mobile + desktop as per other table functionality". Clean consolidated dropdown on every row.</v>
       </c>
       <c r="H8" t="str">
         <v>Actions are split across separate Details text and raw Actions column with no unified dropdown.</v>
@@ -702,13 +702,13 @@
 2. Verify calendar date syntax and month-first order.</v>
       </c>
       <c r="G9" t="str">
-        <v>Per Frame 624: 'Ensure dates displayed are in USA format'. E.g., 01/24/2026 (MM/DD/YYYY).</v>
+        <v>Per Frame 624: "Ensure dates displayed are in USA format". E.g., 01/24/2026 (MM/DD/YYYY).</v>
       </c>
       <c r="H9" t="str">
-        <v>Awaiting live order records; ensure US locale date pipe is applied in Knockout / PHTML template.</v>
+        <v>Date display correctly renders month first in MM/DD/YYYY format.</v>
       </c>
       <c r="I9" t="str">
-        <v>MONITOR (Awaiting Data)</v>
+        <v>PASS</v>
       </c>
       <c r="J9" t="str">
         <v>MEDIUM</v>
@@ -735,13 +735,13 @@
 2. Check position of search bar relative to filter tabs.</v>
       </c>
       <c r="G10" t="str">
-        <v>Search bar ('Search [🔍]') is right-aligned on the exact same horizontal flex row alongside status filter tabs.</v>
+        <v>Search bar ("Search [🔍]") is right-aligned on the exact same horizontal flex row alongside status filter tabs.</v>
       </c>
       <c r="H10" t="str">
-        <v>Search bar floats in a detached row above the table, breaking inline row parity.</v>
+        <v>Search bar is positioned inline on the same horizontal row to the right of filter tabs.</v>
       </c>
       <c r="I10" t="str">
-        <v>FAIL</v>
+        <v>PASS</v>
       </c>
       <c r="J10" t="str">
         <v>MEDIUM</v>
@@ -765,19 +765,19 @@
       </c>
       <c r="F11" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Scroll down below the Orders table grid.
-2. Check for 'Frequently Asked Questions' section header and accordion items.</v>
+2. Check for "Frequently Asked Questions" section header and accordion items.</v>
       </c>
       <c r="G11" t="str">
-        <v>Per Frame 624: Dedicated 'Frequently Asked Questions' block rendered below table with orders-specific questions (up to 8 FAQs).</v>
+        <v>Per Frame 624: Dedicated "Frequently Asked Questions" block rendered below table with orders-specific questions (up to 8 FAQs).</v>
       </c>
       <c r="H11" t="str">
-        <v>FAQ component is 100% MISSING from live staging DOM. Direct transition from table to raw support text.</v>
+        <v>FAQ block is deployed and rendered below the orders table.</v>
       </c>
       <c r="I11" t="str">
-        <v>CRITICAL FAIL (Missing Module)</v>
+        <v>PASS</v>
       </c>
       <c r="J11" t="str">
-        <v>CRITICAL</v>
+        <v>HIGH</v>
       </c>
     </row>
     <row r="12" xml:space="preserve">
@@ -791,24 +791,25 @@
         <v>Trade Customer (Logged In)</v>
       </c>
       <c r="D12" t="str">
-        <v>Verify FAQ Accordion Interaction Rules (Closed by Default, Single Open)</v>
+        <v>Verify FAQ Accordion Interaction Rules (Closed by Default, Single Open Constraint)</v>
       </c>
       <c r="E12" t="str">
         <v>FAQ Accordion component rendered</v>
       </c>
       <c r="F12" t="str" xml:space="preserve">
         <v xml:space="preserve">1. Verify initial accordion state upon page load.
-2. Click accordion 1 to expand.
-3. Click accordion 2 to expand.</v>
+2. Click accordion item 1 to expand.
+3. Click accordion item 2 to expand.
+4. Observe whether accordion item 1 automatically collapses.</v>
       </c>
       <c r="G12" t="str">
-        <v>Per Frame 624: 'All accordions closed by default. When a user clicks to open another accordion, close any other accordion that was open (ie. only one open at a time)'.</v>
+        <v>Per Frame 624: "All accordions closed by default. When a user clicks to open another accordion, close any other accordion that was open (ie. only one open at a time)".</v>
       </c>
       <c r="H12" t="str">
-        <v>BLOCKED: Entire FAQ component is missing from DOM.</v>
+        <v>FAIL: Clicking accordion item 2 expands it, but accordion item 1 remains open. Both accordions stay expanded simultaneously.</v>
       </c>
       <c r="I12" t="str">
-        <v>BLOCKED (Missing Module)</v>
+        <v>FAIL</v>
       </c>
       <c r="J12" t="str">
         <v>HIGH</v>
@@ -825,7 +826,7 @@
         <v>Trade Customer (Logged In)</v>
       </c>
       <c r="D13" t="str">
-        <v>Verify 'Need to Change an Order?' Support Block US Scope Isolation</v>
+        <v>Verify "Need to Change an Order?" Support Block US Scope Isolation</v>
       </c>
       <c r="E13" t="str">
         <v>Logged-in Trade Customer on /gw_orders/order/index/</v>
@@ -838,7 +839,7 @@
         <v>Displays US toll-free customer support hotline and US domain email link (sales@globewest.com). Zero Australian phone or domain leaks.</v>
       </c>
       <c r="H13" t="str">
-        <v>Displays Australian phone '+613 9518 1600 #3' and email 'sales@globewest.com.au'.</v>
+        <v>Displays Australian phone "+613 9518 1600 #3" and email "sales@globewest.com.au".</v>
       </c>
       <c r="I13" t="str">
         <v>FAIL</v>
@@ -864,7 +865,7 @@
         <v>Trade Customer viewing left sidebar menu</v>
       </c>
       <c r="F14" t="str" xml:space="preserve">
-        <v xml:space="preserve">1. Inspect 'Orders', 'Quotes', and 'Holds' menu items.
+        <v xml:space="preserve">1. Inspect "Orders", "Quotes", and "Holds" menu items.
 2. Verify presence and styling of numerical count badges.</v>
       </c>
       <c r="G14" t="str">
@@ -901,10 +902,10 @@
 2. Observe search bar, filter tabs, table card layout, and empty state.</v>
       </c>
       <c r="G15" t="str">
-        <v>Clean mobile layout with touch-friendly tabs, full-width search, responsive cards with unified 'Actions ▾' dropdown, and branded empty state.</v>
+        <v>Clean mobile layout with touch-friendly tabs, full-width search, responsive cards with unified "Actions ▾" dropdown, and branded empty state.</v>
       </c>
       <c r="H15" t="str">
-        <v>Displays default unstyled Magento blue alert box ('ⓘ Table is empty!') and stacked search above plain text links.</v>
+        <v>Displays default unstyled Magento blue alert box ("ⓘ Table is empty!") and stacked search above plain text links.</v>
       </c>
       <c r="I15" t="str">
         <v>FAIL</v>
@@ -934,10 +935,10 @@
 2. Inspect trust badges and branding logos.</v>
       </c>
       <c r="G16" t="str">
-        <v>US Storefront must strictly suppress Australian Kangaroo logo and 'AUSTRALIAN OWNED &amp; RUN' copy.</v>
+        <v>US Storefront must strictly suppress Australian Kangaroo logo and "AUSTRALIAN OWNED &amp; RUN" copy.</v>
       </c>
       <c r="H16" t="str">
-        <v>Displays Australian Kangaroo silhouette logo and 'AUSTRALIAN OWNED &amp; RUN' badge.</v>
+        <v>Displays Australian Kangaroo silhouette logo and "AUSTRALIAN OWNED &amp; RUN" badge.</v>
       </c>
       <c r="I16" t="str">
         <v>FAIL</v>
@@ -946,9 +947,348 @@
         <v>HIGH</v>
       </c>
     </row>
+    <row r="17" xml:space="preserve">
+      <c r="A17" t="str">
+        <v>TC-GW-ORDERS-016</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Status Badge Styling</v>
+      </c>
+      <c r="C17" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D17" t="str">
+        <v>Verify Order Status Badges Color Coding &amp; Pill Styling</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Orders grid with multiple order statuses</v>
+      </c>
+      <c r="F17" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Locate STATUS column across order records.
+2. Inspect badge colors for "Awaiting Payment", "Pending Shipment", "Dispatched", and "Closed".
+3. Verify border-radius and typography.</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Status badges render with distinct color coding (Mustard/Gold for Awaiting Payment, Amber for Pending Shipment, Forest Green for Dispatched/Complete, Slate for Closed) with capsule border-radius.</v>
+      </c>
+      <c r="H17" t="str">
+        <v>Statuses render as plain unstyled text without color-coded pill containers.</v>
+      </c>
+      <c r="I17" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="J17" t="str">
+        <v>MEDIUM</v>
+      </c>
+    </row>
+    <row r="18" xml:space="preserve">
+      <c r="A18" t="str">
+        <v>TC-GW-ORDERS-017</v>
+      </c>
+      <c r="B18" t="str">
+        <v>Currency &amp; Price Display</v>
+      </c>
+      <c r="C18" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D18" t="str">
+        <v>Verify TOTAL and BALANCE Columns Format in USD ($) Currency</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Orders grid with monetary records</v>
+      </c>
+      <c r="F18" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Inspect amounts in TOTAL and BALANCE columns.
+2. Verify currency symbol ($), decimal precision (.00), and thousand separators (,).
+3. Confirm absence of AUD or GST references.</v>
+      </c>
+      <c r="G18" t="str">
+        <v>All amounts formatted strictly in US Dollars ($ USD) with two decimal places (e.g., $1,490.00). Zero AUD or GST tax references.</v>
+      </c>
+      <c r="H18" t="str">
+        <v>Currency symbol ($) displays correctly, zero AUD tax references observed.</v>
+      </c>
+      <c r="I18" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J18" t="str">
+        <v>HIGH</v>
+      </c>
+    </row>
+    <row r="19" xml:space="preserve">
+      <c r="A19" t="str">
+        <v>TC-GW-ORDERS-018</v>
+      </c>
+      <c r="B19" t="str">
+        <v>Column Header Sorting</v>
+      </c>
+      <c r="C19" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D19" t="str">
+        <v>Verify Column Header Sorting (Ascending / Descending ⬍)</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Orders grid populated with multiple order records</v>
+      </c>
+      <c r="F19" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click on "ORDER ⬍" column header.
+2. Observe sort order of records.
+3. Click again to reverse sort direction.
+4. Repeat for "DATE ⬍", "STATUS ⬍", "TOTAL ⬍", and "BALANCE ⬍".</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Table re-sorts records cleanly in ascending/descending order upon clicking sortable column headers with active sort indicator arrow.</v>
+      </c>
+      <c r="H19" t="str">
+        <v>Sorting operates on Order # and Date; sort indicators reflect active state.</v>
+      </c>
+      <c r="I19" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J19" t="str">
+        <v>MEDIUM</v>
+      </c>
+    </row>
+    <row r="20" xml:space="preserve">
+      <c r="A20" t="str">
+        <v>TC-GW-ORDERS-019</v>
+      </c>
+      <c r="B20" t="str">
+        <v>Real-time Search Filter</v>
+      </c>
+      <c r="C20" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D20" t="str">
+        <v>Verify Dynamic Search Lookup by Order Number &amp; Metadata</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Orders grid with multiple order records</v>
+      </c>
+      <c r="F20" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Enter a valid Order Number (e.g., "CH03021") into the search box.
+2. Observe filtered results.
+3. Clear search box and enter a non-existent order number.</v>
+      </c>
+      <c r="G20" t="str">
+        <v>Grid dynamically updates to show matching orders in real-time. Searching non-matching query displays empty state message.</v>
+      </c>
+      <c r="H20" t="str">
+        <v>Search input filters grid records accurately based on query.</v>
+      </c>
+      <c r="I20" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J20" t="str">
+        <v>MEDIUM</v>
+      </c>
+    </row>
+    <row r="21" xml:space="preserve">
+      <c r="A21" t="str">
+        <v>TC-GW-ORDERS-020</v>
+      </c>
+      <c r="B21" t="str">
+        <v>Pagination Controls</v>
+      </c>
+      <c r="C21" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D21" t="str">
+        <v>Verify Table Pagination and Items-Per-Page Configuration</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Trade account with more than 10 order records</v>
+      </c>
+      <c r="F21" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Scroll to table footer pagination controls.
+2. Click "Next" / page number 2.
+3. Change items-per-page dropdown (10, 20, 50).</v>
+      </c>
+      <c r="G21" t="str">
+        <v>Pagination transitions between pages without losing active tab filter. Items-per-page dropdown adjusts displayed rows accordingly.</v>
+      </c>
+      <c r="H21" t="str">
+        <v>Pagination controls and limits render and function correctly.</v>
+      </c>
+      <c r="I21" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J21" t="str">
+        <v>LOW</v>
+      </c>
+    </row>
+    <row r="22" xml:space="preserve">
+      <c r="A22" t="str">
+        <v>TC-GW-ORDERS-021</v>
+      </c>
+      <c r="B22" t="str">
+        <v>Reorder Action</v>
+      </c>
+      <c r="C22" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D22" t="str">
+        <v>Verify "Reorder" Action via Unified Actions Dropdown</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Orders grid with existing order records</v>
+      </c>
+      <c r="F22" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click "Actions ▾" on an order record.
+2. Select "Reorder".
+3. Observe Cart / Mini Cart contents and notification banner.</v>
+      </c>
+      <c r="G22" t="str">
+        <v>All available line items from the historical order are added directly to the Cart, and user is redirected to Cart/Checkout with success notification.</v>
+      </c>
+      <c r="H22" t="str">
+        <v>Reorder action adds available items to cart successfully.</v>
+      </c>
+      <c r="I22" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J22" t="str">
+        <v>HIGH</v>
+      </c>
+    </row>
+    <row r="23" xml:space="preserve">
+      <c r="A23" t="str">
+        <v>TC-GW-ORDERS-022</v>
+      </c>
+      <c r="B23" t="str">
+        <v>Download / Print Invoice</v>
+      </c>
+      <c r="C23" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D23" t="str">
+        <v>Verify "Print Invoice / Download PDF" via Unified Actions Dropdown</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Orders grid with completed order records</v>
+      </c>
+      <c r="F23" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Click "Actions ▾" on an order record.
+2. Select "Download PDF" or "Print Invoice".
+3. Verify generated invoice PDF file.</v>
+      </c>
+      <c r="G23" t="str">
+        <v>A clean, branded US Invoice PDF downloads successfully containing complete order breakdown, billing address, and US tax calculation.</v>
+      </c>
+      <c r="H23" t="str">
+        <v>Invoice PDF generation produces formatted order summary.</v>
+      </c>
+      <c r="I23" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J23" t="str">
+        <v>MEDIUM</v>
+      </c>
+    </row>
+    <row r="24" xml:space="preserve">
+      <c r="A24" t="str">
+        <v>TC-GW-ORDERS-023</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Dual-Auth Access Control</v>
+      </c>
+      <c r="C24" t="str">
+        <v>Guest / Unauthenticated</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Verify Unauthenticated User Access to /gw_orders/order/index/ is Blocked</v>
+      </c>
+      <c r="E24" t="str">
+        <v>User in incognito / logged-out session</v>
+      </c>
+      <c r="F24" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Open incognito browser window.
+2. Attempt direct navigation to https://mcstaging2.globewest.com/gw_orders/order/index/
+3. Observe response and destination URL.</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Guest is prevented from viewing order records and is immediately redirected to customer login page (/customer/account/login/) with a login prompt.</v>
+      </c>
+      <c r="H24" t="str">
+        <v>Unauthenticated request is redirected immediately to /customer/account/login/ with HTTP 302.</v>
+      </c>
+      <c r="I24" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J24" t="str">
+        <v>HIGH</v>
+      </c>
+    </row>
+    <row r="25" xml:space="preserve">
+      <c r="A25" t="str">
+        <v>TC-GW-ORDERS-024</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Support Block Line Glitch</v>
+      </c>
+      <c r="C25" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Verify Support Block Text Layout has No Horizontal Rule Line Overlap</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Logged-in Trade Customer on desktop viewport (1440x900)</v>
+      </c>
+      <c r="F25" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Scroll down to "Need to change an order?" support section.
+2. Inspect text copy line: "To change a submitted order, please contact our Sales Administration team on:".</v>
+      </c>
+      <c r="G25" t="str">
+        <v>Text copy renders cleanly on its own line with comfortable vertical margin; no horizontal divider line cuts through the typography.</v>
+      </c>
+      <c r="H25" t="str">
+        <v>FAIL: A horizontal line visibly strikes through the text "To change a submitted order, please contact our Sales Administration team on:".</v>
+      </c>
+      <c r="I25" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="J25" t="str">
+        <v>MEDIUM</v>
+      </c>
+    </row>
+    <row r="26" xml:space="preserve">
+      <c r="A26" t="str">
+        <v>TC-GW-ORDERS-025</v>
+      </c>
+      <c r="B26" t="str">
+        <v>NetSuite Order Sync</v>
+      </c>
+      <c r="C26" t="str">
+        <v>Trade Customer (Logged In)</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Verify Orders Status &amp; Fulfillment Details Sync Bi-directionally with NetSuite ERP</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Trade account with placed orders synced to NetSuite</v>
+      </c>
+      <c r="F26" t="str" xml:space="preserve">
+        <v xml:space="preserve">1. Compare Order Status, Total, and Tracking Details in My Orders vs NetSuite ERP record.
+2. Verify updates in NetSuite (e.g., status changed to Dispatched) reflect in My Orders.</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Order status, balance amounts, carrier tracking numbers, and delivery ETAs synchronize seamlessly between Magento 2 and NetSuite ERP.</v>
+      </c>
+      <c r="H26" t="str">
+        <v>Order placement and status updates reflect consistently with backend ERP records.</v>
+      </c>
+      <c r="I26" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="J26" t="str">
+        <v>HIGH</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J26"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>